<commit_message>
Monte Carlo del precio objetivo (10.000 iteraciones, semilla 42) con figuras V16/V17; se eliminan las probabilidades de escenarios; notas del Excel actualizadas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0188QZHBkA8n5QL7BtmFakQg
</commit_message>
<xml_diff>
--- a/secciones/valuacion/modelos/Mallplaza_Valoracion_Consolidada_v4_ESG.xlsx
+++ b/secciones/valuacion/modelos/Mallplaza_Valoracion_Consolidada_v4_ESG.xlsx
@@ -117,7 +117,7 @@
     <t xml:space="preserve">NUEVO · v3: hojas TIR_Implicita (TIR de la firma, tasa única, Buscar objetivo) y TIR_Accionista (TIR de la firma, del accionista y por escenario, nominal y real, fórmulas vivas).</t>
   </si>
   <si>
-    <t xml:space="preserve">NUEVO · v3: sin cambios en las demás hojas (valores idénticos a v2). El 7,57% de TIR_Implicita es una tasa única; el 7,56% de la Figura 34/V6 desplaza en paralelo la WACC de cada período.</t>
+    <t xml:space="preserve">NUEVO · v3: sin cambios en las demás hojas (valores idénticos a v2). El 7,61% de TIR_Implicita es una tasa única; el 7,60% de la Figura 27 desplaza en paralelo la WACC de cada período.</t>
   </si>
   <si>
     <t xml:space="preserve">NUEVO · v4: pipeline completo con fecha (170.200 m², USD 613 MM): se activan los «Otros proyectos Chile» (46.500 m², apertura 2028, USD 134 MM) en el forecast (Exhibits v7) y Supuestos!B73 = 114.400 m²; cambian Forecast_Base (filas 5, 7 y 12), el mix de la expansión y, por fórmula, DCF, Deuda, TIR y Sensibilidad.</t>
@@ -2145,7 +2145,7 @@
     <t xml:space="preserve">Chequeo: con C4 = WACC del modelo por período el valor da el valor DCF de la hoja DCF (CLP 1.859); aquí se usa una tasa única para todos los períodos y el terminal.</t>
   </si>
   <si>
-    <t xml:space="preserve">Lectura: quien compra a CLP 3.555 obtiene esta rentabilidad si se cumplen nuestros flujos; es la "WACC implícita en el precio" de las Figuras 28 y 33.</t>
+    <t xml:space="preserve">Lectura: quien compra a CLP 3.555 obtiene esta rentabilidad si se cumplen nuestros flujos; es la "WACC implícita en el precio" de las Figuras 21 y 27 (7,61% tasa única; 7,60% con la curva de WACC desplazada).</t>
   </si>
   <si>
     <t xml:space="preserve">TIR del accionista y de la firma · nominal CLP y real (UF)</t>
@@ -2403,7 +2403,7 @@
     <t xml:space="preserve">Chequeo: valor por acción del DCF con esa tasa (CLP); debe igualar el precio de mercado</t>
   </si>
   <si>
-    <t xml:space="preserve">Chequeo: diferencia con la hoja TIR_Implicita!C4 (pb); la V6 del informe desplaza toda la curva de WACC (7,56%), aquí es una tasa única (7,57%)</t>
+    <t xml:space="preserve">Chequeo: diferencia con la hoja TIR_Implicita!C4 (pb); la Figura 27 del informe desplaza toda la curva de WACC (7,60%), aquí es una tasa única (7,61%)</t>
   </si>
   <si>
     <t xml:space="preserve">E. TIR DEL ACCIONISTA (distribuciones + valor de salida; TIR() trimestral anualizada)</t>

</xml_diff>